<commit_message>
update on SSDI rebuttal and its readme
</commit_message>
<xml_diff>
--- a/SSDI_rebuttal/inference_results.xlsx
+++ b/SSDI_rebuttal/inference_results.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>Dataset</t>
   </si>
@@ -79,6 +79,12 @@
   </si>
   <si>
     <t>74.60 (61.80)</t>
+  </si>
+  <si>
+    <t>93.30 (88.43)</t>
+  </si>
+  <si>
+    <t>73.02 (59.91)</t>
   </si>
   <si>
     <t>* first number is detection accuracy, second number in parenthesis is detection rate, decided based on best_score = 0.5 * num_tn + 0.5 * num_tp (equal weight to tn and tp samples)</t>
@@ -104,12 +110,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -118,11 +130,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -422,21 +437,27 @@
       <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="F4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>